<commit_message>
spacing fixing in note
</commit_message>
<xml_diff>
--- a/output/hadise bornito-test/book-output-list-format-test.xlsx
+++ b/output/hadise bornito-test/book-output-list-format-test.xlsx
@@ -533,7 +533,7 @@
       <c r="E3" s="3" t="inlineStr">
         <is>
           <t>&lt;div class="page-text"&gt;&lt;ar&gt;أَشْهَدُ أَنْ لَّا إِلَهَ إِلَّا اللهُ، وَحْدَهُ لَا شَرِيكَ لَهُ، وَأَشْهَدُ أَنَّ مُحَمَّدًا عَبْدُهُ وَرَسُوْلُهُ، اللَّهُمَّ اجْعَلْنِي مِنَ التَّوَّাবِينَ وَاجْعَلْنِي مِنَ الْمُتَطَهِّرِينَ.&lt;/ar&gt;
-&lt;pronunciation&gt;উচ্চারণ: 'আশহাদু আল্ লা- ইলা-হা ইল্লাল্লা-হু, ওয়াহ্দাহু লা- শারীকা লাহু, ওয়া আশহাদু আন্না মুহাম্মাদান 'আব্দুহু ওয়া রাসূলুহু, আল্লা-হুম্মাজ্ 'আল্লী মিনাৎ তাওয়া-বীনা ওয়াজ 'আল্লী মিনাল্ মুতাত্বাহিরীন'&lt;/pronunciation&gt;
+&lt;pronunciation&gt;উচ্চারণ: 'আশহাদু আল্ লা- ইলা-হা ইল্লাল্লা-হু, ওয়াহ্দাহু লা- শারীকা লাহু, ওয়া আশহাদু আন্না মুহাম্মাদান 'আব্দুহু ওয়া রাসূলুহু, আল্লা-হুম্মাজ্ 'আল্নী মিনাৎ তাওয়া-বীনা ওয়াজ 'আল্নী মিনাল্ মুতাত্বাহিরীন'&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'আমি সাক্ষ্য দিচ্ছি আল্লাহ তা'আলা ব্যতীত আর কোন সত্য ইলাহ নেই, তিনি একক, তাঁর কোন শরীক নেই; আমি আরো সাক্ষ্য দিচ্ছি মুহাম্মাদ (ﷺ) তাঁর বান্দা ও রাসূল। হে আল্লাহ! আমাকে তাওবাকারীদের অন্তর্ভুক্ত করুন এবং আমাকে পবিত্রতা অর্জনকারীদের অন্তর্ভুক্ত করুন'&lt;/meaning&gt;
 &lt;p&gt;উমার ইবনুল খাত্তাব (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) বলেছেন, যে ব্যক্তি সুন্দরভাবে অযু করার পর এই দু'আ পাঠ করবে, তার জন্য জান্নাতের আটটি দরজাই খুলে দেয়া হবে। সে নিজ ইচ্ছায় যে কোন দরজা দিয়েই তাতে প্রবেশ করতে পারবে। [৮২]&lt;/p&gt;
 &lt;p&gt;ব্যাখ্যা: হাদীসে অযুর পর পঠিতব্য যে দু'আটি উল্লেখ করা হয়েছে তার দ্বারা মূলত আল্লাহর সন্তুষ্টির লক্ষ্যে করা আমলের স্বচ্ছতা ও হাদীসে আব্বার ও আসগার থেকে অঙ্গ-প্রত্যঙ্গের পবিত্রতা লাভের পর অন্তরকে শিরক ও রিয়া থেকে পবিত্র রাখার দিকে ইশারা করা হয়েছে। তাওবাহ গোপন গুনাহ হতে পবিত্রকারী এবং অযু আল্লাহর নৈকট্য অর্জনে বাধাদানকারী বাহ্যিক গুনাহের পবিত্রকারী। হাদীসে বলা হয়েছে, 'যে ব্যক্তি পূর্ণাঙ্গভাবে অযু করার পর শাহাদাতায়ন পাঠ করে, তার জন্য জান্নাতের আটটি দরজা খুলে দেয়া হয়'। এ বক্তব্যের মর্মার্থ হচ্ছে, ব্যক্তি জান্নাতে প্রবেশ করতে চাইলে একটি দরজাই তার জন্য যথেষ্ট, তথাপিও হাদীসে জান্নাতের আটটি দরজা খুলে দেয়ার কথা বলা হয়েছে। এটি মূলত ব্যক্তির কর্মের সম্মানার্থে।&lt;/p&gt;&lt;br&gt;&lt;div class="subheading"&gt;অযুর শেষে পাঠ করার দু'আ&lt;/div&gt;&lt;br&gt;&lt;p&gt;অথবা বাহ্যিক দৃষ্টিভঙ্গির দিকে দৃষ্টি দিলে বলা যায়, ব্যক্তি যে ধরনের আমল বেশি করবে তার জন্য ঐ আমলের প্রস্তুত করা বিশেষ দরজা খুলে দেয়া হবে। কারণ জান্নাতের দরজাসমূহ প্রস্তুত করা হয়েছে বিশেষ বিশেষ আমলের জন্য। যেমন- যে ব্যক্তি বেশি বেশি সিয়াম (রোযা) পালন করবে তার জন্য জান্নাতের 'রাইয়্যান' [৮৩] নামক দরজা খুলে দেয়া হবে। অনুরূপ যে ব্যক্তি যেমন আমল করবে তাঁর জন্য তেমন দরজা খুলে দেয়া হবে। ইবনু সাইয়্যিদিন নাস বলেন, দরজার সংখ্যাধিক্যতা খুলে দেয়া ও এসব হতে ডাকা ইত্যাদি ক্বিয়ামতের দিন ব্যক্তির সম্মান এবং মর্যাদার দিকেই ইশারা। অতএব বিষয়টি এমন নয় যে, কোন এক দরজা দিয়ে ডাকা হলে সে দরজার সীমা সে অতিক্রম করবে না। বরং প্রত্যেক দরজা দিয়ে ডাক পাওয়ার পর যে দরজা দিয়ে ইচ্ছা সে দরজা দিয়েই সে প্রবেশ করবে। [৮৪]&lt;/p&gt;&lt;br&gt;&lt;div class="subheading"&gt;আরেকটি দু'আ:&lt;/div&gt;&lt;br&gt;&lt;ar&gt;سُبْحَانَكَ اللَّهُمَّ وَبِحَمْدِكَ، أَشْهَدُ أَنْ لَّا إِلَهَ إِلَّا أَنْتَ، أَسْتَغْفِرُكَ وَأَتُوبُ إِلَيْكَ.&lt;/ar&gt;
@@ -572,13 +572,13 @@
         <is>
           <t>&lt;div class="page-text"&gt;&lt;p&gt;আবু সাঈদ আল খুদরী (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) বলেন, যখন তোমরা আযান শুনতে পাও তখন মুয়াযযিন যা বলে তোমরাও তা-ই বলো। [৮৬] শুধু&lt;/p&gt;
 &lt;ar&gt;حَيَّ عَلَى الصَّلَاةِ، حَيَّ عَلَى الْفَلَاحِ.&lt;/ar&gt;
-&lt;pronunciation&gt;উচ্চারণ: 'হাঁইয়া 'আলাস্থ স্বলা-হ, হাঁইয়া 'আলাল্ ফালা-হ'&lt;/pronunciation&gt;
+&lt;pronunciation&gt;উচ্চারণ: 'হাঁইয়া 'আলাস্ স্বলা-হ, হাঁইয়া 'আলাল্ ফালা-হ'&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'এসো স্বলাতের দিকে, এসো কল্যাণের দিকে'&lt;/meaning&gt;
 &lt;p&gt;এর সময়ে বলবে,&lt;/p&gt;
 &lt;ar&gt;لَا حَوْলَ وَلَا قُوَّةَ إِلَّا بِاللَّهِ.&lt;/ar&gt;
 &lt;pronunciation&gt;উচ্চারণ: লা- হাঁওলা ওয়ালা- কুওয়াতা ইল্লা বিল্লা-হ'&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'আল্লাহর সাহায্য ছাড়া (পাপ কাজ থেকে দূরে থাকার) কোন উপায় এবং (সৎকাজ করার) কোন শক্তি কারো নেই'। [৮৭]&lt;/meaning&gt;
-&lt;p&gt;ব্যাখ্যা: কেউ যদি দূরত্ব অথবা অন্ধত্বের কারণে মুয়াযয্যিনের শব্দ শুনতে না পায়, তাহলে তার জন্য আযানের উত্তর দেয়ার বিধান প্রযোজ্য নয়। মুয়াযয্যিনের আযানের জবাবে শ্রোতারা তাই বলবে যা মুয়াযযিন বলে। তবে দুই 'হাইয়্যা 'আলা স্বলাহ'-এর لَا حَوْলَ وَلَا قُوَّةَ إِلَّا بِاللَّهِ ('লা হাওলা ওয়ালা- কুউওয়াতা ইল্লা- বিল্লা-হ') বলবে। আর এটা উমার (রাঃ)-এর বর্ণিত হাদীসে রয়েছে। আর ফজরের আযানের সময় মুয়াযযিন যখন الصَّلَاةُ خَيْرُ مِّنَ النَّوْমِ বলেন, তখন এর উত্তরে صَدَّقْتَ وَবَرَرْتَ বলার কোন দলীল পাওয়া যায় না। [৮৮]&lt;/p&gt;&lt;/div&gt;</t>
+&lt;p&gt;ব্যাখ্যা: কেউ যদি দূরত্ব অথবা অন্ধত্বের কারণে মুয়াযযিনের শব্দ শুনতে না পায়, তাহলে তার জন্য আযানের উত্তর দেয়ার বিধান প্রযোজ্য নয়। মুয়াযযিনের আযানের জবাবে শ্রোতারা তাই বলবে যা মুয়াযযিন বলে। তবে দুই 'হাইয়্যা 'আলা স্বলাহ'-এর لَا حَوْলَ وَلَا قُوَّةَ إِلَّا بِاللَّهِ ('লা হাওলা ওয়ালা- কুউওয়াতা ইল্লা- বিল্লা-হ') বলবে। আর এটা উমার (রাঃ)-এর বর্ণিত হাদীসে রয়েছে। আর ফজরের আযানের সময় মুয়াযযিন যখন الصَّلَاةُ خَيْرُ مِّنَ النَّوْমِ বলেন, তখন এর উত্তরে صَدَّقْتَ وَবَرَرْتَ বলার কোন দলীল পাওয়া যায় না। [৮৮]&lt;/p&gt;&lt;/div&gt;</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -609,7 +609,7 @@
       <c r="E5" s="3" t="inlineStr">
         <is>
           <t>&lt;div class="page-text"&gt;&lt;ar&gt;اللَّهُمَّ رَبَّ هَذِهِ الدَّعْوَةِ التَّামَّةِ، وَالصَّلَاةِ الْقَائِمَةِ ، أتِ مُحَمَّدًا الْوَسِيْلَةَ وَالْفَضِيلَةَ، وَابْعَثْهُ مَقَامًا মَّحْمُوْডًا الَّذِي وَعَدْتَهُ.&lt;/ar&gt;
-&lt;pronunciation&gt;উচ্চারণ: 'আল্লা-হুম্মা রব্বা হা-যিহিদ্ দা'ওয়াতিৎ তা-ম্মাতি, ওয়াস্ স্বলা- তিল্ ক্ব-য়িমাহ, আ-তি মুহাম্মাদাল্ ওয়াসীলাতা ওয়াল্ ফাদ্বীলাতা, ওয়ার্ 'আহ্হু মাক্বা-মাম্ মাহমূদাল্ লাযী ওয়া 'আদ্রাহ'&lt;/pronunciation&gt;
+&lt;pronunciation&gt;উচ্চারণ: 'আল্লা-হুম্মা রব্বা হা-যিহিদ্ দা'ওয়াতিৎ তা-ম্মাতি, ওয়াস্ স্বলা- তিল্ ক্ব-য়িমাহ, আ-তি মুহাম্মাদাল্ ওয়াসীলাতা ওয়াল্ ফাদ্বীলাতা, ওয়াব্'আছ্হু মাক্বা-মাম্ মাহমূদাল্ লাযী ওয়া'আদ্তাহ'&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'হে আল্লাহ! এ পরিপূর্ণ আহ্বান ও প্রতিষ্ঠিত স্বালাতের মালিক, মুহাম্মাদ (ﷺ)-কে ওয়াসীলা ও সর্বোচ্চ মর্যাদার অধিকারী করুন এবং তাঁকে সে 'মাকামে মাহমুদ'-এ পৌঁছে দিন যার অঙ্গীকার আপনি করেছেন'&lt;/meaning&gt;
 &lt;p&gt;জাবির ইবনু আব্দুল্লাহ (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) বলেছেন, যে ব্যক্তি আযান শুনে এই দু'আ পাঠ করবে, ক্বিয়ামতের দিন সে আমার শাফা'আত লাভের অধিকারী হবে। [৮৯]&lt;/p&gt;
 &lt;p&gt;ব্যাখ্যা: আযানের জবাব দেয়ার পর দু'আ পড়ার পূর্বে দুরূদ পাঠ করা মুস্তাহাব। ওয়াসীলা হলো জান্নাতের একটি বিশেষ স্থান, যা রাসূল (ﷺ)-এর জন্য নির্ধারিত। আযানের শেষে এই ওয়াসীলা যোগ করে দু'আ করলে নবীর শাফা'আত পাবার আশা করা যায়। 'যখন আযান শেষ হবে'- এখানে শেষ হওয়ার সাধারণ অর্থ হলো, আযান যখন পূর্ণ হয়। আর এর প্রমাণ আবদুল্লাহ ইবনু আমর ইবনুল আস (রাঃ)-এর বর্ণিত হাদীস। আযান শেষ হলে আযানের দু'আ পড়বে। ইমাম হাফিয (রাহঃ)-এর মতে উক্ত দু'আর মধ্যকার দা'ওয়াত দ্বারা উদ্দেশ্য হলো- একত্ববাদের দিকে ডাকা। যে আহ্বানের মধ্যে কোন শিরক নেই। এ প্রসঙ্গে সূরা রা'দ-এর ১৪নং আয়াতে বলা হয়েছে, لَهُ دَعْوَةُ الْحَقِّ অর্থাৎ- 'আল্লাহর জন্যই সত্যের দিকে আহ্বান'। উক্ত দু'আর একটি অংশ وَالصَّلَاةِ الْقَائِمَةِ (ওয়াস্ব স্বলা- তিল্ ক্ব-য়িমাহ) এর উদ্দেশ্য হল- ক্বিয়ামত পর্যন্ত এ স্বলাত (নামায) ক্বায়িম থাকবে।&lt;/p&gt;
@@ -619,9 +619,9 @@
 &lt;ar&gt;مَنْ تَعَمَّدَ عَلَى كَذِبًا فَلْيَتَبَوَّأْ مَقْعَدَهُ مِنَ النَّارِ&lt;/ar&gt;
 &lt;p&gt;'আমার নামে মিথ্যারোপ করলো, সে জাহান্নামে তার ঠিকানা বানিয়ে নিলো'। অত্র হাদীসের শেষাংশে [১] 'ইন্নাকা লা তুখলিফুল মী'আদ। [২] বায়হাক্বীতে (১ম খণ্ডের ৪১০ পৃষ্ঠা) বর্ণিত আযানের দু'আর শুরুতে 'আল্লাহুম্মা ইন্নী আস-আলুকা বি হাক্কি হা-যিহিদ দা'ওয়াতি। [৩] ইমাম তাহাভীর শারহু মা'আনিল আসার-এ বর্ণিত 'আ-তি সাইয়্যিদিনা মুহাম্মাদান। [৪] ইবনুস সুন্নীর 'ফী 'আমালিল ইয়াওমি ওয়াল লায়লাহ' গ্রন্থে ওয়াদ দারাজাতার রাফী'আহ। [৫] রাফী'ঈ প্রণীত 'আল মুহাররির গ্রন্থে আযানের দু'আর শেষে বর্ণিত 'ইয়া আরহামার রা-হিমীন। আযানের জওয়াবে প্রচলিত বাড়তি বিষয়গুলো অবশ্যই পরিত্যাজ্য। অতিরিক্ত শব্দগুলো সহীহ সূত্রে প্রমাণিত নয়। রেডিও এবং বাংলাদেশ টেলিভিশন থেকে প্রচারিত দু'আয় 'ওয়ারযুকনা শা'আতাহু ইয়াওমাল ক্বিয়ামাহ' বাক্যটি যা যোগ করা হয়েছে&lt;/p&gt;
 &lt;p&gt;তার কোন ভিত্তি নেই।&lt;/p&gt;&lt;br&gt;&lt;div class="subheading"&gt;আরেকটি দু'আ:&lt;/div&gt;&lt;br&gt;&lt;ar&gt;لَا إِلَهَ إِلَّا اللَّهُ وَحْدَهُ لَا شَرِيكَ لَهُ وَأَنَّ مُحَمَّدًا عَبْدُهُ وَرَسُوْلُهُ، رَضِيتُ بِاللَّهِ رَبًّا وَبِمُحَمَّدٍ رَسُوْلًا وَبِالْإِسْلَامِ دِينًا.&lt;/ar&gt;
-&lt;pronunciation&gt;উচ্চারণ: 'লা- ইলা-হা ইল্লাল্লা-হু, ওয়াহ্দাহু লা- শারীকা লাহু, ওয়া আন্না মুহাম্মাদান 'আব্দুহু ওয়া রাসূলুহু, রাদ্বীতু বিল্লা-হি রব্বান, ওয়া বিমুহাম্মাদিন রাসূলান, ওয়া বিল্টুস্লা-মি দীনান'।&lt;/pronunciation&gt;
+&lt;pronunciation&gt;উচ্চারণ: 'লা- ইলা-হা ইল্লাল্লা-হু, ওয়াহ্দাহু লা- শারীকা লাহু, ওয়া আন্না মুহাম্মাদান 'আব্দুহু ওয়া রাসূলুহু, রাদ্বীতু বিল্লা-হি রব্বান, ওয়া বিমুহাম্মাদিন রাসূলান, ওয়া বিল্ ইস্লা-মি দীনান'।&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'আল্লাহ ছাড়া প্রকৃত কোন ইলাহ নেই। তিনি একক, তাঁর কোন শরীক নেই। আমি আরো সাক্ষ্য দিচ্ছি যে, মুহাম্মাদ আল্লাহর বান্দা ও রাসূল। আমি আল্লাহকে রব, ইসলামকে দ্বীন এবং মুহাম্মাদ-কে রাসূল হিসেবে পেয়ে সন্তুষ্ট'।&lt;/meaning&gt;
-&lt;p&gt;সা'দ ইবনু আবী ওয়াক্কাস (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) বলেছেন, যে ব্যক্তি মুয়াযয্যিনের আযান শুনে এই দু'আ পড়বে, তার সমস্ত গুনাহ ক্ষমা করে দেয়া হবে। [৯৩]&lt;br&gt;&lt;br&gt;ব্যাখ্যা: এ হাদীসে আযানের পর আল্লাহর একত্ববাদ ও নবী (ﷺ)-এর রিসালাতের সাক্ষ্য দান এবং একটি বিশেষ দু'আর মাহাত্ম্য ও ফযীলত বর্ণনা করা হয়েছে। আযানের জবাব দিলে শাহাদাতায়ন এর বাক্য উচ্চারণ করতে হয়। এ বিষয়টি বিশেষ গুরুত্বপূর্ণ বিধায় আযানের জবাবের পর পৃথকভাবে তাওহীদ ও রিসালাতের সাক্ষ্যের বিষয় উল্লেখ করা হয়েছে। শাহাদাতের বাক্যের পর যে দু'আটি উল্লেখ করা হয়েছে তাতে বলা হয়েছে যে, আল্লাহকে রব হিসেবে পেয়ে সন্তুষ্ট থাকা, অর্থাৎ তাঁর রবুবিয়্যাতের সকল বিষয়ের উপর সন্তুষ্ট থাকা। আল্লাহ কর্তৃক নির্ধারিত বিষয়কে নিজের জন্য কল্যাণকর হিসেবে মেনে নেয়া। মুহাম্মাদ (ﷺ)-কে রাসূল হিসেবে মেনে নেয়ার অর্থ তিনি বিশ্বাসগত এবং 'আমালগত যেসব বিষয় নিয়ে আগমন করেছেন, তার সব কিছুকেই মেনে নেয়া। ইসলামকে পেয়ে সন্তুষ্ট হওয়ার অর্থ হলো-&lt;/p&gt;&lt;/div&gt;</t>
+&lt;p&gt;সা'দ ইবনু আবী ওয়াক্কাস (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) বলেছেন, যে ব্যক্তি মুয়াযযিনের আযান শুনে এই দু'আ পড়বে, তার সমস্ত গুনাহ ক্ষমা করে দেয়া হবে। [৯৩]&lt;br&gt;&lt;br&gt;ব্যাখ্যা: এ হাদীসে আযানের পর আল্লাহর একত্ববাদ ও নবী (ﷺ)-এর রিসালাতের সাক্ষ্য দান এবং একটি বিশেষ দু'আর মাহাত্ম্য ও ফযীলত বর্ণনা করা হয়েছে। আযানের জবাব দিলে শাহাদাতায়ন এর বাক্য উচ্চারণ করতে হয়। এ বিষয়টি বিশেষ গুরুত্বপূর্ণ বিধায় আযানের জবাবের পর পৃথকভাবে তাওহীদ ও রিসালাতের সাক্ষ্যের বিষয় উল্লেখ করা হয়েছে। শাহাদাতের বাক্যের পর যে দু'আটি উল্লেখ করা হয়েছে তাতে বলা হয়েছে যে, আল্লাহকে রব হিসেবে পেয়ে সন্তুষ্ট থাকা, অর্থাৎ তাঁর রবুবিয়্যাতের সকল বিষয়ের উপর সন্তুষ্ট থাকা। আল্লাহ কর্তৃক নির্ধারিত বিষয়কে নিজের জন্য কল্যাণকর হিসেবে মেনে নেয়া। মুহাম্মাদ (ﷺ)-কে রাসূল হিসেবে মেনে নেয়ার অর্থ তিনি বিশ্বাসগত এবং 'আমালগত যেসব বিষয় নিয়ে আগমন করেছেন, তার সব কিছুকেই মেনে নেয়া। ইসলামকে পেয়ে সন্তুষ্ট হওয়ার অর্থ হলো-&lt;/p&gt;&lt;/div&gt;</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -655,14 +655,14 @@
         <is>
           <t>&lt;div class="page-text"&gt;&lt;p&gt;ইসলামের সকল আদেশ-নিষেধ ও বিধি-বিধানকে সন্তুষ্টচিত্তে মেনে নেয়া ও এসবের বিরুদ্ধাচরণ না করা। [৯৪]&lt;/p&gt;&lt;br&gt;&lt;div class="subheading"&gt;মসজিদে প্রবেশের দু'আ&lt;/div&gt;&lt;br&gt;&lt;p&gt;সর্বপ্রথম রাসূল (ﷺ)-এর উপর দুরূদ পাঠ করবে। অতঃপর বলবে,&lt;/p&gt;
 &lt;ar&gt;اللَّهُمَّ افْتَحْ لِي أَبْوَابَ رَحْمَتِكَ.&lt;/ar&gt;
-&lt;pronunciation&gt;উচ্চারণ: 'আল্লা-হুম্মাফ্ তালী আওয়া-বা রহমাতিকা'।&lt;/pronunciation&gt;
+&lt;pronunciation&gt;উচ্চারণ: 'আল্লা-হুম্মাফ্ তাহ্লী আব্ওয়া-বা রহমাতিকা'।&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'হে আল্লাহ! আপনার রহমতের দরজা আমার জন্য খুলে দিন'।&lt;/meaning&gt;
 &lt;p&gt;আব্দুল মালিক ইবনু সাঈদ ইবনু সুওয়াইদ বলেন, আমি আবূ উসাইদ আনসারী (রাঃ)-কে বলতে শুনেছি, রাসূলুল্লাহ (ﷺ) বলেছেন, তোমাদের কেউ মসজিদে প্রবেশের সময় যেন সর্বপ্রথম আমার উপর দুরূদ পাঠ করে, অতঃপর এই দু'আ বলে। [৯৫]&lt;br&gt;&lt;br&gt;ব্যাখ্যা: যখন মাসজিদে প্রবেশ করবে তখন اللَّهُمَّ افْتَحْ لِي أَبْوَابَ رَحْمَتِكَ পাঠ করবে। আবূ দাউদ-এর বর্ণনায় এসেছে, প্রথমে রাসূল (ﷺ)-এর প্রতি সালাম ও দুরূদ পাঠ করবে, পরে এ দু'আটি পাঠ করবে। ইমাম নাবাবী (রাহিমাহুল্লাহ) বলেন, এই দু'আ পাঠ করা মুস্তাহাব। ইবনু মাজাহ-এর বর্ণনায় এসেছে,&lt;/p&gt;
 &lt;ar&gt;بِسْمِ اللَّهِ ، وَالسَّلَامُ عَلَى رَسُولِ اللهِ ، اَللَّهُمَّ اغْفِرْ لِي ذُنُوبِي وَافْتَحْ لِي أَبْوَابَ رَحْمَتِكَ.&lt;/ar&gt;
-&lt;pronunciation&gt;উচ্চারণ: 'বিস্মিল্লা-হি, ওয়াস্সালা-মু 'আলা- রাসূলিল্লা-হ, আল্লা-হুম্মাগ্ ফির লী যুনূবী ওয়াস্তাহ্ লী আওয়া-বা রাহুঁমাতিক'।&lt;/pronunciation&gt;
+&lt;pronunciation&gt;উচ্চারণ: 'বিস্মিল্লা-হি, ওয়াস্সালা-মু 'আলা- রাসূলিল্লা-হ, আল্লা-হুম্মাগ্ ফির লী যুনূবী ওয়াফ্তাহ্ লী আব্ওয়া-বা রাহ্মাতিকা'।&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'আল্লাহর নামে (প্রবেশ) এবং আল্লাহর রাসূলকে সালাম। হে আল্লাহ!&lt;/meaning&gt;
 &lt;p&gt;আমার গুনাহসমূহ ক্ষমা করুন এবং আমার জন্য আপনার রহমতের (দয়ার) দরজাসমূহ উন্মুক্ত করে দিন'। ফাতিমাহ (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) মসজিদে প্রবেশকালে এই দু'আ বলতেন। [৯৭]&lt;/p&gt;&lt;br&gt;&lt;div class="subheading"&gt;আরেকটি দু'আ:&lt;/div&gt;&lt;br&gt;&lt;ar&gt;أَعُوْذُ بِاللَّهِ الْعَظِيمِ وَبِوَجْهِهِ الْكَرِيمِ وَসُلْطَانِهِ الْقَدِيمِ مِنَ الشَّيْطَانِ الرَّجِيمِ.&lt;/ar&gt;
-&lt;pronunciation&gt;উচ্চারণ: 'আয়ূযু বিল্লা-হিল্ 'আযীমি ওয়া বিওয়াহহিল্ কারীমি ওয়া সুত্ত্বা-নিহিল্ ক্বদীমি মিনাশ শাইত্বা-নির্ রাজীম'।&lt;/pronunciation&gt;
+&lt;pronunciation&gt;উচ্চারণ: 'আয়ূযু বিল্লা-হিল্ 'আযীমি ওয়া বিওয়াজ্হিহিল্ কারীমি ওয়া সুল্ত্বা-নিহিল্ ক্বদীমি মিনাশ শাইত্বা-নির্ রাজীম'।&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'আমি মহান আল্লাহর মর্যাদাপূর্ণ চেহারা ও তাঁর অফুরন্ত ক্ষমতায় বিতাড়িত শয়তান থেকে আশ্রয় প্রার্থনা করছি'।&lt;/meaning&gt;
 &lt;p&gt;• হাইওয়াহ ইবনু শুরায়িহ (রাহিমাহুল্লাহ) বলেন, আমি উক্ববাহ ইবনু মুসলিমের সাথে সাক্ষাৎ করে বলি, আমি জানতে পারলাম যে, আপনার নিকট আব্দুল্লাহ ইবনু আমর ইবনুল আস (রাঃ)-এর মাধ্যমে নবী (ﷺ) হতে বর্ণিত হয়েছে, নবী (ﷺ) মসজিদে প্রবেশের সময় উপরোক্ত দু'আ বলতেন। উক্ববাহ (রাঃ) বললেন, 'এতটুকুই?' আমি বললাম, 'হ্যাঁ'। উক্ববাহ (রাঃ) বললেন, 'কেউ এ দু'আ পাঠ করলে শয়তান বলে, এ লোকটি আমার (অনিষ্ট ও কুমন্ত্রণা) থেকে সারা দিনের জন্য বেঁচে গেল'। [৯৮]&lt;br&gt;&lt;br&gt;ব্যাখ্যা: রাসূলুল্লাহ (ﷺ) মসজিদে প্রবেশের জন্য এর দরজায় পৌঁছলে এ দু'আ পড়তেন। তিনি আরো বলেন, যখন কোন মু'মিন এই দু'আ পড়ে তখন শয়তান বলে- 'এই দু'আকারী আমার পথভ্রষ্টতা থেকে দিনের বাকী সময় বা সারা দিন-রাত রক্ষা পেল'। [৯৯]&lt;/p&gt;&lt;/div&gt;</t>
         </is>
@@ -698,7 +698,7 @@
       <c r="E7" s="3" t="inlineStr">
         <is>
           <t>&lt;div class="page-text"&gt;&lt;ar&gt;اللَّهُمَّ إِنِّي أَسْأَلُكَ مِنْ فَضْلِكَ&lt;/ar&gt;
-&lt;pronunciation&gt;উচ্চারণ: 'আল্লা-হুম্মা ইন্নী আলুকা মিং ফালিকা'।&lt;/pronunciation&gt;
+&lt;pronunciation&gt;উচ্চারণ: 'আল্লা-হুম্মা ইন্নী আস্আলুকা মিং ফাদ্বলিকা'।&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'হে আল্লাহ! আপনার কাছে আপনার অনুগ্রহ প্রার্থনা করছি'।&lt;/meaning&gt;
 &lt;p&gt;আবূ উসাঈদ (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) বলেছেন, তোমাদের কেউ যখন মসজিদ থেকে বের হবে তখন এই দু'আ পড়বে। [১০০]&lt;br&gt;&lt;br&gt;ব্যাখ্যা: প্রবেশের সময় রহমতকে এবং বের হওয়ার সময় অনুগ্রহকে নির্ধারণ করার কারণ হলো- রহমত আল্লাহর কিতাবে আত্মিক ও মানসিক প্রশান্তির নি'আমত এবং পরকালের নি'আমত। যেমন- আল্লাহ তা'আলা বলেন,&lt;/p&gt;
 &lt;ar&gt;رَحْمَتُ رَبِّكَ خَيْرٌ مِّمَّا يَجْمَعُونَ&lt;/ar&gt;
@@ -709,12 +709,12 @@
 &lt;p&gt;অর্থাৎ, 'সালাত সমাপ্ত হলে তোমরা পৃথিবীতে ছড়িয়ে পড়ো এবং আল্লাহর অনুগ্রহ সন্ধান করো'। [১০০] যে মাসজিদে প্রবেশ করবে সে আল্লাহর নৈকট্য কামনা করবে। এমন কাজে ব্যস্ত হবে যা প্রতিদান ও জান্নাতের নিকটবর্তী করবে। সুতরাং তা রহমত ও দু'আর সাথে সংশ্লিষ্ট। আর বের হওয়াটা হলো রিযিক বা যাবতীয় প্রয়োজন। এজন্য অনুগ্রহ দু'আর সাথে সংশ্লিষ্ট। [১০৪]&lt;/p&gt;
 &lt;p&gt;ইবনু মাজাহ-এর বর্ণনায় এসেছে,&lt;/p&gt;
 &lt;ar&gt;بِسْمِ اللَّهِ ، وَالسَّلَامُ عَلَى رَسُولِ اللهِ ، اللَّهُمَّ اغْفِرْ لِي ذُنُوبِي وَافْتَحْ لِي أَبْوَابَ فَضْلِكَ.&lt;/ar&gt;
-&lt;pronunciation&gt;উচ্চারণ: 'বিস্মিল্লা-হি, ওয়াস্সালা-মু 'আলা- রাসূলিল্লা-হ, আন্ন আল্লা-হুম্মাগ্ ফির লী যুনূবী ওয়াস্তাহ্ লী আওয়া-বা ফালিকা'&lt;/pronunciation&gt;
+&lt;pronunciation&gt;উচ্চারণ: 'বিস্মিল্লা-হি, ওয়াস্সালা-মু 'আলা- রাসূলিল্লা-হ, আল্লা-হুম্মাগ্ ফির লী যুনূবী ওয়াফ্তাহ্ লী আব্ওয়া-বা ফাদ্বলিকা'&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'আল্লাহর নামে (প্রবেশ) এবং আল্লাহর রাসূলকে সালাম। হে আল্লাহ! আমার গুনাহসমূহ ক্ষমা করুন এবং আমার জন্য আপনার অনুগ্রহের দরজাসমূহ উন্মুক্ত করে দিন'&lt;/meaning&gt;
 &lt;p&gt;ফাতিমাহ (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) প্রবেশকালে এই দু'আ বলতেন। [১০৫]&lt;/p&gt;
 &lt;p&gt;মসজিদে আরেকটি দু'আ:&lt;/p&gt;
 &lt;ar&gt;اللَّهُمَّ اعْصِمْنِي مِنَ الشَّيْطَانِ الرَّحِيْمِ.&lt;/ar&gt;
-&lt;pronunciation&gt;উচ্চারণ: 'আল্লা-হুম্মা' মিনাশ্ শাইত্ব-নির্ রাজীম'&lt;/pronunciation&gt;
+&lt;pronunciation&gt;উচ্চারণ: 'আল্লা-হুম্মা'সিম্নী মিনাশ্ শাইত্ব-নির্ রাজীম'&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'হে আল্লাহ! আমাকে বিতাড়িত শয়তান থেকে রক্ষা করুন'&lt;/meaning&gt;
 &lt;p&gt;আবূ হুরাইরাহ (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) মসজিদ থেকে বের হতে এই দু'আ পাঠ করতে বলেছেন। [১০৬]&lt;/p&gt;&lt;/div&gt;</t>
         </is>
@@ -752,14 +752,14 @@
         <is>
           <t>&lt;div class="page-text"&gt;&lt;div class="subheading"&gt;সানা (তাক্বীরে তাহরীমার পর পঠিতব্য)&lt;/div&gt;&lt;br&gt;&lt;ar&gt;( اللَّهُمَّ بَاعِدْ بَيْنِي وَالْمَاءِ وَالْبَرَدِ ..... ) :&lt;/ar&gt;
 &lt;ar&gt;اللَّهُمَّ بَاعِدْ بَيْنِي وَبَيْنَ خَطَايَايَ كَمَا بَاعَدْتَ بَيْنَ الْمَشْرِقِ وَالْمَغْرِبِ اللَّهُمَّ نَقِنِي مِنْ خَطَايَايَ كَمَا يُنَقَّى الثَّوْبُ الْأَبْيَضُ مِنَ الدَّنَسِ، اَللَّهُمَّ اغْسِلْنِي مِنْ خَطَايَايَ بِالثَّلْجِ وَالْمَاءِ وَالْبَرَدِ.&lt;/ar&gt;
-&lt;pronunciation&gt;উচ্চারণ: 'আল্লা-হুম্মা বা-ঈদ বাইনী ওয়া বাইনা খাত্ত্বা-ইয়া-ইয়া কামা বা-'আস্তা বাইনাল্ মাশ্রিক্কি ওয়াল্ মাগ্রিব, আল্লা-হুম্মা নাক্বক্বিনী মিন খাত্বা-ইয়া-ইয়া কামা ইউনাক্বক্বাহ্ ছাওবুল্ আইয়াদু মিনাদ্ দানাস, আল্লা-হুম্মাগ্‌ সিল্কী মিন খাত্ত্বা-ইয়া-ইয়া বিছাল্লিল্ল্জ ওয়াল্ মা-য়ি ওয়াল্ বারাদ'&lt;/pronunciation&gt;
+&lt;pronunciation&gt;উচ্চারণ: 'আল্লা-হুম্মা বা-ঈদ বাইনী ওয়া বাইনা খাত্ত্বা-ইয়া-ইয়া কামা বা-'আস্তা বাইনাল্ মাশ্রিক্কি ওয়াল্ মাগ্রিব, আল্লা-হুম্মা নাক্বক্বিনী মিন খাত্বা-ইয়া-ইয়া কামা ইউনাক্বক্বাহ্ ছাওবুল্ আইয়াদু মিনাদ্ দানাস, আল্লা-হুম্মাগ্‌ সিল্কী মিন খাত্ত্বা-ইয়া-ইয়া বিছাল্জি ওয়াল্ মা-য়ি ওয়াল্ বারাদ'&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'হে আল্লাহ আমার ও আমার পাপের মাঝে এতটা দূরত্ব সৃষ্টি করে দিন, যেমন পশ্চিম ও পূর্বের মধ্যে আপনি দূরত্ব রেখেছেন। হে আল্লাহ! আমাকে আমার পাপ থেকে এমনভাবে পরিষ্কার করে দিন, যেমনভাবে সাদা কাপড় থেকে ময়লা পরিষ্কার করা হয়। হে আল্লাহ! আপনি আমার পাপসমূহ বরফ, পানি ও তুষারের শুভ্রতা দ্বারা ধুয়ে পরিষ্কার করে দিন'&lt;/meaning&gt;
-&lt;p&gt;আবূ হুরাইরাহ (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) স্বলাত শুরু করলে তাব্বীরে তাহরীমা (আল্লাহু আব্বার) বলে কিরা'আত শুরু করার আগে কিছুক্ষণ চুপ থাকতেন। এ দেখে আমি জিজ্ঞেস করলাম, 'হে আল্লাহর রাসূল! আমার পিতা-মাতা আপনার জন্য কুরবান হোক! আপনি স্বলাতের তাব্বীরে তাহরীমা ও কিরা'আতের মাঝে যখন চুপ থাকেন তখন কি পড়েন?' রাসূলুল্লাহ (ﷺ) আমাকে তখন এই দু'আর কথা বললেন। [১০৭]&lt;/p&gt;
+&lt;p&gt;আবূ হুরাইরাহ (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) স্বলাত শুরু করলে তাকবীরে তাহরীমা (আল্লাহু আকবার) বলে কিরা'আত শুরু করার আগে কিছুক্ষণ চুপ থাকতেন। এ দেখে আমি জিজ্ঞেস করলাম, 'হে আল্লাহর রাসূল! আমার পিতা-মাতা আপনার জন্য কুরবান হোক! আপনি স্বলাতের তাকবীরে তাহরীমা ও কিরা'আতের মাঝে যখন চুপ থাকেন তখন কি পড়েন?' রাসূলুল্লাহ (ﷺ) আমাকে তখন এই দু'আর কথা বললেন। [১০৭]&lt;/p&gt;
 &lt;p&gt;ব্যাখ্যা: এটা তাকবীর ও ক্বিরাআতের মধ্যে দু'আ পড়ার সুন্নাত প্রকাশ পায়। এক্ষেত্রে 'সুব্‌হাঁ-নাকা আল্লা-হুম্মা ওয়া বিহাঁদিক.....' পড়া সুন্নাত। ইমাম মালিক&lt;/p&gt;
 &lt;p&gt;ও আহমাদ (রাহিমাহুল্লাহ)-এর প্রকাশ্য মাযহাবও অনুরূপ। ইমাম আবূ ইউসুফ (রাহিমাহুল্লাহ)-এর মতে 'ইন্নী ওয়াজ্জাহতু ওয়াহিয়া লিল্লাযী....' এ দু'আ উভয়টি পড়া সুন্নাত। হানাফীরা দু'আগুলো নফল ও তাহাজ্জুদ স্বলাতে সাব্যস্ত করে সুন্নাত বলেন। এ ধরনের মন্তব্য সঠিক নয়। রাসূল (ﷺ) সানা পড়ার ক্ষেত্রে ফরয ও নফলের মধ্যে কোন পার্থক্য করেনি। তাই সব স্বলাতেই দু'আ পড়া যাবে। [১০৮]&lt;/p&gt;
 &lt;ar&gt;( وَجَّهْتُ وَجْهِيَ ... وَأَتُوْبُ إِلَيْكَ : )&lt;/ar&gt;
 &lt;ar&gt;وَجَّهْتُ وَجْهِيَ لِلَّذِي فَطَرَ السَّمَوتِ وَالْأَرْضَ حَنِيفًا وَمَا أَنَا مِنَ الْمُشْرِكِينَ، إِنَّ صَلَاتِي وَنُسُكِي وَمَحْيَايَ وَمَمَاتِي لِلَّهِ رَبِّ الْعَالَمِينَ، لَا شَرِيكَ لَهُ وَبِذَلِكَ أُمِرْتُ وَأَنَا مِنَ الْمُسْلِمِينَ، اَللَّهُمَّ أَنْتَ الْمَلِكُ لَا إِلَهَ إِلَّا أَنْتَ، أَنْتَ رَبِّي وَأَنَا عَبْدُكَ ظَلَمْتُ نَفْسِيْ وَاعْتَرَفْتُ بِذَنْبِي فَاغْفِرْ لِي ذُنُوبِي جَمِيْعًا إِنَّهُ لَا يَغْفِرُ الذُّنُوبَ إِلَّا أَنْتَ، وَاهْدِنِي لْأَحْسَنِ الْأَخْلَاقِ لَا يَهْدِي لَأَحْسَنِهَا إِلَّا أَنْتَ، وَاصْرِفْ عَنِّي سَيِّئَهَا لَا يَصْرِفُ عَنِّي سَيِّهَا إِلَّا أَنْتَ، لَبَّيْكَ وَسَعْدَيْكَ وَالْخَيْرُ كُلُّهُ فِي يَدَيْكَ وَالشَّرُّ لَيْسَ إِلَيْكَ أَنَا بِكَ وَإِلَيْكَ تَبَارَكْتَ وَتَعَالَيْتَ اَسْتَغْفِرُكَ وَأَتُوْبُ إِلَيْكَ.&lt;/ar&gt;
-&lt;pronunciation&gt;উচ্চারণ: 'ওয়াজ্জাহ্ ওয়াহিয়া লিল্লাযী ফাত্মারাস্ সামা-ওয়া-তি ওয়াল্ আরদ্বা হাঁনীফাও ওয়ামা- আনা- মিনাল মুশ্রিকীন, ইন্না স্বলা-তী ওয়া নুসুকী ওয়া মাহঁইয়া-ইয়া ওয়া মামা-তী লিল্লা-হি রব্বিল্ 'আ-লামীন, লা- শারীকা লাহু ওয়া বিযালিকা উমিরত ওয়া আনা- মিনাল্ মুস্লিমীন, আল্লা-হুম্মা আংতাল্ মালিকু লা- ইলা-হা ইল্লা- আংতা, আংতা রব্বী ওয়া আনা- 'আব্দুকা লাড্ডু নাসী ওয়া'তারা বিযানী ফাফির্ লী যুনূবী জামী'আন ইন্নাহu লা- ইয়াগফিরুয যুনুবা ইল্লা- আংতা, ওয়াদিনীল্ আহ্সানিল্ আল্লা- লা- ইয়াহ্দীল্ আহ্সানিহা- ইল্লা- আংতা, ওয়াস্রিফ 'আন্নী সাইয়্যিআহা- লা- ইয়াম্ব্রিফু 'আন্নী সাইয়্যিআহা- ইল্লা- আংতা, লাব্বাইকা ওয়া সা'দাইকা ওয়াল্ খইরু কুল্লাহু ফী ইয়াদাইকা ওয়াশ্ শারু লাইসা ইলাইকা আনা- বিকা, ওয়া ইলাইকা তাবা-রাক্কা ওয়া তা'আ-&lt;/pronunciation&gt;
+&lt;pronunciation&gt;উচ্চারণ: 'ওয়াজ্জাহ্তু ওয়াজ্হিয়া লিল্লাযী ফাত্মারাস্ সামা-ওয়া-তি ওয়াল্ আরদ্বা হাঁনীফাও ওয়ামা- আনা- মিনাল মুশ্রিকীন, ইন্না স্বলা-তী ওয়া নুসুকী ওয়া মাহঁইয়া-ইয়া ওয়া মামা-তী লিল্লা-হি রব্বিল্ 'আ-লামীন, লা- শারীকা লাহু ওয়া বিযালিকা উমিরতু ওয়া আনা- মিনাল্ মুস্লিমীন, আল্লা-হুম্মা আংতাল্ মালিকু লা- ইলা-হা ইল্লা- আংতা, আংতা রব্বী ওয়া আনা- 'আব্দুকা যালামতু নাফ্সী ওয়া'তারাফ্তু বিযাম্বী ফাগ্ফির্ লী যুনূবী জামী'আন ইন্নাহu লা- ইয়াগফিরুয যুনুবা ইল্লা- আংতা, ওয়াদিনীল্ আহ্সানিল্ আখ্লা-ক্বি লা- ইয়াহ্দীল্ আহ্সানিহা- ইল্লা- আংতা, ওয়াস্রিফ 'আন্নী সাইয়্যিআহা- লা- ইয়াস্রিফু 'আন্নী সাইয়্যিআহা- ইল্লা- আংতা, লাব্বাইকা ওয়া সা'দাইকা ওয়াল্ খইরু কুল্লাহু ফী ইয়াদাইকা ওয়াশ্ শারু লাইসা ইলাইকা আনা- বিকা, ওয়া ইলাইকা তাবা-রক্তা ওয়া তা'আ-&lt;/pronunciation&gt;
 &lt;pronunciation&gt;লাইতা আস্তাগফিরুকা ওয়া আতুবু ইলাইক'&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'আমি একনিষ্ঠ হয়ে আমার মুখ সে মহান সত্ত্বার দিকে ফিরিয়ে নিলাম যিনি আসমান ও যমীনকে সৃষ্টি করেছেন। আর আমি মুশরিকদের অন্তর্ভুক্ত নই। আমার স্বলাত, আমার কুরবানী, আমার জীবন ও মৃত্যু সবকিছুই আল্লাহর জন্য যিনি সারা বিশ্বজাহানের প্রতিপালক। তাঁর কোন শরীক নেই। আমি এ জন্যই আদিষ্ট হয়েছি। আমি মুসলিম বা আত্মসমর্পণকারী। হে আল্লাহ! আপনিই সার্বভৌম বাদশাহ। আপনি ছাড়া আর কোন সত্য ইলাহ নেই। আপনি আমার প্রতিপালক, আর আমি আপনার বান্দা। আমি নিজে আমার প্রতি যুলুম করেছি। আমি আমার পাপ স্বীকার করছি। সুতরাং আপনি আমার সব পাপ ক্ষমা করে দিন। কেননা আপনি ছাড়া আর কেউ পাপ ক্ষমা করতে পারে না। আমাকে সর্বোত্তম আখলাক বা নৈতিকতার পথ দেখান। আপনি ছাড়া এ পথ আর কেউ দেখাতে সক্ষম নয়। আর আখলাক বা নৈতিকতার মন্দ দিকগুলো আমার থেকে দূরে রাখুন। আপনি ছাড়া আর কেউ মন্দগুলোকে দূরে রাখতে সক্ষম নয়। আমি আপনার সামনে হাজির আছি, আপনার আনুগত্য করতে প্রস্তুত আছি। সব রকম কল্যাণের মালিক আপনিই। অকল্যাণের দায়-দায়িত্ব আপনার নয়। আমার সব কামনা-বাসনা আপনার কাছেই কাম্য। আমার শক্তিসামর্থ্যও আপনারই দেয়া। আপনি কল্যাণময়, আপনি মহান। আমি আপনার কাছে ক্ষমা প্রার্থনা করছি এবং আপনার কাছেই তাওবাহ করছি'&lt;/meaning&gt;
 &lt;p&gt;আলী ইবনু আবূ ত্বালিব (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) যখন স্বলাত আদায় করতেন তখন এই দু'আ দ্বারা স্বলাত শুরু করতেন। [১০৯]&lt;br&gt;&lt;br&gt;ব্যাখ্যা: যেহেতু রাসূলুল্লাহ (ﷺ) কোন স্বলাতকে নির্দিষ্ট করেননি, সেহেতু সকল স্বলাতে দু'আ-যিক্রগুলো পড়া সুন্নাতরীতি হিসেবে পরিগণিত হবে। সহীহ মুসলিমের সহীহ হাদীসটি রাতের স্বলাতের ব্যাপারে নাযিল হয়েছে। তবে তা এ নির্দেশ করে না যে, দু'আ-আযকারগুলো রাতের তাহাজ্জুদ স্বলাতের জন্যে নির্দিষ্ট। মুহাম্মাদ ইবনু&lt;/p&gt;
@@ -771,7 +771,7 @@
 &lt;p&gt;আয়িশাহ (রাঃ) সূত্রে বর্ণিত, রাসূলুল্লাহ (ﷺ) স্বলাত (নামায) আরম্ভকালে এই দু'আ পড়তেন। [১১২]&lt;br&gt;&lt;br&gt;ব্যাখ্যা: এ দু'আটি পড়া সহীহ সূত্রে প্রমাণিত। আবু হুরাইরাহ (রাঃ) বর্ণিত হাদীসও যে বিশুদ্ধ, তা সন্দেহাতীত। তবে আবূ দাঊদ-এর সানাদটি সহীহ বিধায় এর উপর আমল করা যায়। উমার (রাঃ) এটা পড়তেন যখন অনেক সাহাবা উপস্থিত থাকতেন। তিনি এটা দিয়ে সাহাবীগণের প্রশিক্ষণ দিতেন।&lt;/p&gt;
 &lt;p&gt;শওকানী রাহিমাহুল্লাহ বলেন, যেটা সবচেয়ে বিশুদ্ধ সেটাকে প্রাধান্য দেয়া ও গ্রহণ করা উত্তম হবে।&lt;/p&gt;
 &lt;meaning&gt;অর্থ: 'সুব্‌হাঁ-নাকা আল্লা-হুম্মা ওয়া বিহাঁদিকা' এর অর্থ হলো- 'হে আল্লাহ! আমি আপনার প্রশংসা সম্বলিত চূড়ান্ত ও সর্বোচ্চ পবিত্রতা ঘোষণা করছি, আপনি বরকতময়, আপনার নামে রয়েছে প্রভূত কল্যাণ'। 'ওয়া তা'আ-লা- জাদ্দুকা' এর মানে হলো- 'আমি আপনার আযমত বা বড়ত্বকে সকল কিছুর উপর তুলে ধরছি'। 'ওয়া লা- ইলা-হা গাইরুকা' এর এ অর্থও হতে পারে, আপনি সকল কিছু থেকে অমুখাপেক্ষী এবং আপনার অমুখাপেক্ষীতা সকল কিছু থেকে ঊর্ধ্বে।&lt;/meaning&gt;&lt;br&gt;&lt;div class="subheading"&gt;৮: (أَنْتَ سُبْحَانَكَ ... وَجَّهْتُ وَجْهِيَ لِلَّذِي)&lt;/div&gt;&lt;br&gt;&lt;ar&gt;وَجَّهْتُ وَجْهِيَ لِلَّذِي فَطَرَ السَّمَوتِ وَالْأَرْضَ حَنِيفًا وَمَا أَنَا مِنَ الْمُشْرِكِينَ، اللَّهُمَّ أَنْتَ الْمَلِكُ لَا إِلَهَ إِلَّا أَنْتَ سُبْحَانَكَ.&lt;/ar&gt;
-&lt;pronunciation&gt;উচ্চারণ: 'ওয়াজ্জাহ্ ওয়াহিয়া লিল্লাযী ফাত্মারাস্ সামা-ওয়া-তি ওয়াল্ আর্দ্রা হানীফাও ওয়ামা- আনা- মিনাল্ মুশ্রিকীন, আল্লা-হুম্মা আংতাল্ মালিকু লা- ইলা-হা ইল্লা- আংতা সুব্‌হাঁ-নাকা'&lt;/pronunciation&gt;
+&lt;pronunciation&gt;উচ্চারণ: 'ওয়াজ্জাহ্তু ওয়াজ্হিয়া লিল্লাযী ফাত্মারাস্ সামা-ওয়া-তি ওয়াল্ আরদ্বা হানীফাও ওয়ামা- আনা- মিনাল্ মুশ্রিকীন, আল্লা-হুম্মা আংতাল্ মালিকু লা- ইলা-হা ইল্লা- আংতা সুব্‌হাঁ-নাকা'&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'আমি একনিষ্ঠ হয়ে আমার মুখ সে মহান সত্ত্বার দিকে ফিরিয়ে নিলাম যিনি আসমান ও যমীনকে সৃষ্টি করেছেন। আর আমি মুশরিকদের অন্তর্ভুক্ত নই। হে আল্লাহ! আপনিই বাদশাহ, আপনি ছাড়া সত্যিকার কোন মা'বুদ নেই। আপনি পবিত্র, সকল প্রশংসা আপনার জন্য'&lt;/meaning&gt;
 &lt;p&gt;মুহাম্মাদ ইবনু মাসলামাহ (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) নফল স্বলাত আদায় করতে দাঁড়ালে উক্ত দু'আ পাঠ করতেন। এরপর তিনি (ﷺ) ক্বিরাআত শুরু করতেন। [১১৪]&lt;/p&gt;
 &lt;p&gt;ব্যাখ্যা: মুল্লা আলী আল-ক্বারী রাহিমাহুল্লাহ বলেন, অত্র হাদীসের প্রকাশমান অর্থ এই যে, নফল বা সুন্নাত স্বলাতের প্রারম্ভে 'ওয়াজ্জাহ্ ওয়াছিয়া.....' শেষ&lt;/p&gt;
@@ -814,7 +814,7 @@
 &lt;pronunciation&gt;উচ্চারণ: 'আয়ূযু বিল্লা-হি মিনাশ শাইত্ব-নির্ রাজীম'&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'বিতাড়িত শয়তান থেকে আল্লাহর নিকট আশ্রয় প্রার্থনা করছি'&lt;/meaning&gt;
 &lt;p&gt;উসমান ইবনু আবুল আস (রাঃ) নবী (ﷺ)-এর কাছে এসে বললেন, 'হে আল্লাহর রাসূল! শয়তান আমার, আমার স্বলাত ও কিরা'আতের মধ্যে বাধা হয়ে দাঁড়ায় এবং সবকিছুতে গোলমাল বাধিয়ে দেয়'। তখন রাসূলুল্লাহ (ﷺ) বললেন, 'এটা এক প্রকারের শয়তান- যার নাম 'খিনযিব'। যে সময় তুমি তার উপস্থিতি বুঝতে পারবে, তখন (আয়ূযুবিল্লাহ পড়ে) তার অনিষ্ট হতে আল্লাহর কাছে আশ্রয় চেয়ে তিনবার তোমার বাম পাশে থুথু ফেলবে'&lt;/p&gt;
-&lt;p&gt;তিনি বলেন, 'তারপরে আমি তা করলাম আর আল্লাহ আমার হতে তা দূর করে দিলেন'। [১১৬]&lt;br&gt;&lt;br&gt;ব্যাখ্যা: يُلَبِّسُهَا عَلَيَّ অর্থাৎ, স্বলাতে গোলমাল বাধিয়ে দেয় এবং ক্বিরাআত&lt;/p&gt;&lt;br&gt;&lt;div class="subheading"&gt;৯- ذَاكَ شَيْطَانٌ يُقَالُ لَهُ خِنْزَبٌ&lt;/div&gt;&lt;br&gt;&lt;p&gt;গোলমাল সৃষ্টিকারী একজন বিশেষ শয়তানের নাম খিনযাব। [১১৭]&lt;/p&gt;&lt;/div&gt;</t>
+&lt;p&gt;তিনি বলেন, 'তারপরে আমি তা করলাম আর আল্লাহ আমার হতে তা দূর করে দিলেন'। [১১৬]&lt;br&gt;&lt;br&gt;ব্যাখ্যা: يُلَبِّسُهَا عَلَيَّ অর্থাৎ, স্বলাতে গোলমাল বাধিয়ে দেয় এবং ক্বিরাআত&lt;/p&gt;&lt;br&gt;&lt;div class="subheading"&gt;৯- ذَاكَ شَيْطَانٌ يُقَالُ لَهُ خِنْزَبٌ&lt;/div&gt;&lt;br&gt;&lt;p&gt;গোলমাল সৃষ্টিকারী একজন বিশেষ শয়তানের নাম 'খিনযাব'। [১১৭]&lt;/p&gt;&lt;/div&gt;</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -850,7 +850,7 @@
 &lt;meaning&gt;অর্থ: 'আমি প্রশংসার সাথে আপনার পবিত্রতা বর্ণনা করছি, আপনি ছাড়া কোন সত্য মা'বুদ নেই'&lt;/meaning&gt;
 &lt;p&gt;ইবনু জুরাইয রাহিমাহুল্লাহ হতে বর্ণিত, তিনি বলেন, আমি আতাকে জিজ্ঞেস করলাম, 'আপনি রুকু'তে কি পড়েন?' তিনি বলেন, 'সুবহা-নাকা ওয়া বিহামদিকা লা- ইলা-হা ইল্লা- আংতা'। অর্থাৎ 'হে আল্লাহ! আমরা প্রশংসার সাথে আপনার পবিত্রতা বর্ণনা করছি, আপনি ব্যতীত কোন সত্য মা'বুদ নেই'। কেননা ইবনু আবূ মুলাইকাহ আমাকে আয়িশাহ (রাঃ) সূত্রে অবহিত করেছেন যে, তিনি (আয়িশাহ) বলেন, একরাতে আমি ঘুম থেকে জেগে নবী (ﷺ)-কে আমার কাছে পেলাম না। আমি ধারণা করলাম, তিনি হয়তো তাঁর অপর কোন স্ত্রীর কাছে গেছেন। আমি তাঁর খোঁজে বের হলাম, কিন্তু না পেয়ে ফিরে আসলাম। দেখি, তিনি রুকু' অথবা (রাবীর সন্দেহ) সাজদায় আছেন এবং উক্ত দু'আ বলছেন।&lt;/p&gt;
 &lt;p&gt;আমি বললাম, আমার পিতা-মাতা আপনার জন্য উৎসর্গ হোক। আমি কি ধারণায় নিমজ্জিত হয়েছি, আর আপনি কি কাজে মগ্ন আছেন। [১২১]&lt;/p&gt;&lt;br&gt;&lt;div class="subheading"&gt;(وَعَظْمِي وَعَصَبِي ... اللَّهُمَّ لَكَ رَكَعْتُ)&lt;/div&gt;&lt;br&gt;&lt;ar&gt;اللَّهُمَّ لَكَ رَكَعْتُ وَبِكَ آمَنْتُ وَلَكَ أَسْلَمْتُ خَشَعَ لَكَ سَمْعِي وَبَصَرِي وَمُنِّي وَعَظْمِي وَعَصَبِي.&lt;/ar&gt;
-&lt;pronunciation&gt;উচ্চারণ: 'আল্লা-হুম্মা লাকা রকা'তু, ওয়া বিকা আ-মাংতু, ওয়া বিকা আস্লাম, খশা'আ সাক্ষ্মী ওয়া বাস্বারী ওয়া মুখী ওয়া 'আযী ওয়া 'আস্বাবী'&lt;/pronunciation&gt;
+&lt;pronunciation&gt;উচ্চারণ: 'আল্লা-হুম্মা লাকা রকা'তু, ওয়া বিকা আ-মাংতু, ওয়া বিকা আস্লাম, খশা'আ লাকা সাম্'য়ী ওয়া বাস্বারী ওয়া মুখী ওয়া 'আয্মী ওয়া 'আস্বাবী'&lt;/pronunciation&gt;
 &lt;meaning&gt;অর্থ: 'হে আল্লাহ! আপনার জন্য রুকু করলাম, আপনার উপর ঈমান আনলাম এবং আপনার নিকটেই আত্মসমর্পণ করলাম। আমার কান, চোখ, মগজ, হাড় এবং সব স্নায়ুতন্ত্রী আপনার কাছে নত ও বশীভূত হলো'&lt;/meaning&gt;
 &lt;p&gt;আলী ইবনু আবূ তালিব (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) যখন রুকু'তে যেতেন তখন এই দু'আ পাঠ করতেন। [১২২]&lt;/p&gt;&lt;br&gt;&lt;div class="subheading"&gt;(سُبْحَانَكَ اللَّهُمَّ رَبَّنَا ...)&lt;/div&gt;&lt;br&gt;&lt;ar&gt;سُبْحَانَكَ اللَّهُمَّ رَبَّنَا وَبِحَمْدِكَ، اللَّهُمَّ اغْفِرْ لِي.&lt;/ar&gt;
 &lt;pronunciation&gt;উচ্চারণ: 'সুবহা-নাকা আল্লা-হুম্মা রব্বানা- ওয়া বিহাঁদিকা, আল্লা-হুম্মাগ্ ফির লী'&lt;/pronunciation&gt;

</xml_diff>